<commit_message>
feat: Günlük veriler ve dashboard bileşenlerinde iyileştirmeler yapıldı; yeni testler eklendi, gereksiz kodlar kaldırıldı
</commit_message>
<xml_diff>
--- a/wwwroot/EXCELS/Günlük Çalışma Verileri.xlsx
+++ b/wwwroot/EXCELS/Günlük Çalışma Verileri.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10412"/>
   <workbookPr codeName="BuÇalışmaKitabı"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tuncay/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tuncay/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50CDD5AC-AC1C-254C-BA0C-A8986EB03ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E53489AD-9CB9-6C42-8A82-90AA98909552}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1620" yWindow="1140" windowWidth="29040" windowHeight="14460" tabRatio="898" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21460" tabRatio="898" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Veriler" sheetId="3" r:id="rId1"/>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sayfa1!$A$1:$D$124</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Veriler!$B$1:$R$941</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Veriler!$B$1:$R$1205</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1342" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1386" uniqueCount="144">
   <si>
     <t>Üretime Verilen Parça Sayısı</t>
   </si>
@@ -460,6 +460,15 @@
     <t>İş Gecikmesi(Kurum 2024 DENİZBANK ŞUBE  GÜVENLİK BANKOSU)</t>
   </si>
   <si>
+    <t>İş Gecikmesi(ÖZEL DENİZBANK YENİ TİP GÜVENLİK BANKOSU)</t>
+  </si>
+  <si>
+    <t>İş Gecikmesi(BOYA 2024 ZİRAAT BANKASI  ÜRÜNLERİ)</t>
+  </si>
+  <si>
+    <t>İş Gecikmesi(CNC SPACE MASA VE MASA TABLASI)</t>
+  </si>
+  <si>
     <t>MODUL</t>
   </si>
 </sst>
@@ -470,12 +479,28 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="77" x14ac:knownFonts="1">
+  <fonts count="80" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="162"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="162"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1088,6 +1113,13 @@
       <charset val="162"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -1160,17 +1192,17 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="76" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="78" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="117">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="74" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="76" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="74" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="76" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1178,13 +1210,13 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="74" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="76" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="10" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="4" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="74" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="76" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1192,6 +1224,8 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="75" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="74" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="73" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="72" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="71" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1220,8 +1254,12 @@
     <xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1231,20 +1269,20 @@
     <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1266,28 +1304,22 @@
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="76" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="75" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="74" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1300,22 +1332,22 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1325,40 +1357,46 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1375,16 +1413,17 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="79" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1662,7 +1701,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sayfa1"/>
-  <dimension ref="B1:R1181"/>
+  <dimension ref="B1:R1221"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="12.5" bestFit="1" customWidth="1"/>
@@ -1717,8 +1756,8 @@
       <c r="N1" t="s">
         <v>18</v>
       </c>
-      <c r="O1" t="s">
-        <v>140</v>
+      <c r="O1" s="116" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="2" spans="2:15" x14ac:dyDescent="0.2">
@@ -38088,9 +38127,6 @@
       <c r="L1139" s="17"/>
       <c r="M1139" s="17"/>
       <c r="N1139" s="17"/>
-      <c r="O1139">
-        <v>255</v>
-      </c>
     </row>
     <row r="1140" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B1140" s="5" t="s">
@@ -38675,7 +38711,7 @@
       <c r="M1155" s="17"/>
       <c r="N1155" s="17"/>
       <c r="O1155">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="1156" spans="2:15" x14ac:dyDescent="0.2">
@@ -39402,7 +39438,7 @@
         <v>46119</v>
       </c>
     </row>
-    <row r="1178" spans="2:15" x14ac:dyDescent="0.2">
+    <row r="1178" spans="2:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B1178" s="1" t="s">
         <v>11</v>
       </c>
@@ -39491,7 +39527,7 @@
         <v>4</v>
       </c>
       <c r="H1180" s="4">
-        <f t="shared" ref="H1180:H1181" si="449">D1180/G1180</f>
+        <f t="shared" ref="H1180:H1187" si="449">D1180/G1180</f>
         <v>385.25</v>
       </c>
       <c r="I1180" s="10">
@@ -39532,6 +39568,1477 @@
       <c r="I1181" s="10">
         <v>46119</v>
       </c>
+    </row>
+    <row r="1182" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1182" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1182" s="20">
+        <v>969</v>
+      </c>
+      <c r="D1182" s="20">
+        <v>969</v>
+      </c>
+      <c r="E1182" s="20">
+        <f t="shared" ref="E1182:E1189" si="450">C1182-D1182</f>
+        <v>0</v>
+      </c>
+      <c r="F1182" s="3">
+        <f t="shared" ref="F1182:F1189" si="451">D1182/C1182</f>
+        <v>1</v>
+      </c>
+      <c r="G1182" s="2">
+        <v>5</v>
+      </c>
+      <c r="H1182" s="4">
+        <f t="shared" si="449"/>
+        <v>193.8</v>
+      </c>
+      <c r="I1182" s="10">
+        <v>46120</v>
+      </c>
+      <c r="J1182" s="17">
+        <v>1</v>
+      </c>
+      <c r="K1182" s="17"/>
+      <c r="L1182" s="17"/>
+      <c r="M1182" s="17">
+        <v>11</v>
+      </c>
+      <c r="N1182" s="17"/>
+    </row>
+    <row r="1183" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1183" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1183" s="6">
+        <v>1013</v>
+      </c>
+      <c r="D1183" s="6">
+        <v>883</v>
+      </c>
+      <c r="E1183" s="2">
+        <f t="shared" si="450"/>
+        <v>130</v>
+      </c>
+      <c r="F1183" s="3">
+        <f t="shared" si="451"/>
+        <v>0.87166831194471861</v>
+      </c>
+      <c r="G1183" s="2">
+        <v>9</v>
+      </c>
+      <c r="H1183" s="4">
+        <f t="shared" si="449"/>
+        <v>98.111111111111114</v>
+      </c>
+      <c r="I1183" s="10">
+        <v>46120</v>
+      </c>
+      <c r="J1183" s="17">
+        <v>2</v>
+      </c>
+      <c r="K1183" s="17"/>
+      <c r="L1183" s="17"/>
+      <c r="M1183" s="17"/>
+      <c r="N1183" s="17">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="1184" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1184" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1184" s="2">
+        <v>77</v>
+      </c>
+      <c r="D1184" s="2">
+        <v>77</v>
+      </c>
+      <c r="E1184" s="2">
+        <f t="shared" si="450"/>
+        <v>0</v>
+      </c>
+      <c r="F1184" s="3">
+        <f t="shared" si="451"/>
+        <v>1</v>
+      </c>
+      <c r="G1184" s="2">
+        <v>9</v>
+      </c>
+      <c r="H1184" s="4">
+        <f t="shared" si="449"/>
+        <v>8.5555555555555554</v>
+      </c>
+      <c r="I1184" s="10">
+        <v>46120</v>
+      </c>
+      <c r="J1184" s="17"/>
+      <c r="K1184" s="17"/>
+      <c r="L1184" s="17"/>
+      <c r="M1184" s="17"/>
+      <c r="N1184" s="17"/>
+    </row>
+    <row r="1185" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1185" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1185" s="6">
+        <f>561+405</f>
+        <v>966</v>
+      </c>
+      <c r="D1185" s="99">
+        <f>443+281</f>
+        <v>724</v>
+      </c>
+      <c r="E1185" s="2">
+        <f t="shared" si="450"/>
+        <v>242</v>
+      </c>
+      <c r="F1185" s="3">
+        <f t="shared" si="451"/>
+        <v>0.74948240165631475</v>
+      </c>
+      <c r="G1185" s="6">
+        <v>10</v>
+      </c>
+      <c r="H1185" s="4">
+        <f t="shared" si="449"/>
+        <v>72.400000000000006</v>
+      </c>
+      <c r="I1185" s="10">
+        <v>46120</v>
+      </c>
+      <c r="J1185" s="17">
+        <v>16</v>
+      </c>
+      <c r="K1185" s="17"/>
+      <c r="L1185" s="17"/>
+      <c r="M1185" s="17"/>
+      <c r="N1185" s="17"/>
+    </row>
+    <row r="1186" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1186" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1186" s="20">
+        <v>1168</v>
+      </c>
+      <c r="D1186" s="20">
+        <v>893</v>
+      </c>
+      <c r="E1186" s="2">
+        <f t="shared" si="450"/>
+        <v>275</v>
+      </c>
+      <c r="F1186" s="3">
+        <f t="shared" si="451"/>
+        <v>0.76455479452054798</v>
+      </c>
+      <c r="G1186" s="6">
+        <v>9</v>
+      </c>
+      <c r="H1186" s="4">
+        <f t="shared" si="449"/>
+        <v>99.222222222222229</v>
+      </c>
+      <c r="I1186" s="10">
+        <v>46120</v>
+      </c>
+      <c r="J1186" s="17">
+        <v>2</v>
+      </c>
+      <c r="K1186" s="17">
+        <v>6</v>
+      </c>
+      <c r="L1186" s="17"/>
+      <c r="M1186" s="17"/>
+      <c r="N1186" s="17"/>
+    </row>
+    <row r="1187" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1187" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1187" s="20">
+        <v>209</v>
+      </c>
+      <c r="D1187" s="20">
+        <v>209</v>
+      </c>
+      <c r="E1187" s="2">
+        <f t="shared" si="450"/>
+        <v>0</v>
+      </c>
+      <c r="F1187" s="3">
+        <f t="shared" si="451"/>
+        <v>1</v>
+      </c>
+      <c r="G1187" s="6">
+        <v>16</v>
+      </c>
+      <c r="H1187" s="4">
+        <f t="shared" si="449"/>
+        <v>13.0625</v>
+      </c>
+      <c r="I1187" s="10">
+        <v>46120</v>
+      </c>
+      <c r="J1187" s="17"/>
+      <c r="K1187" s="17"/>
+      <c r="L1187" s="17"/>
+      <c r="M1187" s="17"/>
+      <c r="N1187" s="17"/>
+      <c r="O1187">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="1188" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1188" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1188" s="2">
+        <v>426</v>
+      </c>
+      <c r="D1188" s="6">
+        <v>409</v>
+      </c>
+      <c r="E1188" s="2">
+        <f t="shared" si="450"/>
+        <v>17</v>
+      </c>
+      <c r="F1188" s="3">
+        <f t="shared" si="451"/>
+        <v>0.960093896713615</v>
+      </c>
+      <c r="G1188" s="6">
+        <v>4</v>
+      </c>
+      <c r="H1188" s="4">
+        <f t="shared" ref="H1188:H1195" si="452">D1188/G1188</f>
+        <v>102.25</v>
+      </c>
+      <c r="I1188" s="10">
+        <v>46120</v>
+      </c>
+      <c r="J1188" s="17"/>
+      <c r="K1188" s="17"/>
+      <c r="L1188" s="17">
+        <v>9</v>
+      </c>
+      <c r="M1188" s="17"/>
+      <c r="N1188" s="17">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="1189" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1189" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1189" s="2">
+        <v>285</v>
+      </c>
+      <c r="D1189" s="6">
+        <v>285</v>
+      </c>
+      <c r="E1189" s="2">
+        <f t="shared" si="450"/>
+        <v>0</v>
+      </c>
+      <c r="F1189" s="3">
+        <f t="shared" si="451"/>
+        <v>1</v>
+      </c>
+      <c r="G1189" s="6">
+        <v>2</v>
+      </c>
+      <c r="H1189" s="4">
+        <f t="shared" si="452"/>
+        <v>142.5</v>
+      </c>
+      <c r="I1189" s="10">
+        <v>46120</v>
+      </c>
+      <c r="J1189" s="17"/>
+      <c r="K1189" s="17"/>
+      <c r="L1189" s="17"/>
+      <c r="M1189" s="17"/>
+      <c r="N1189" s="17"/>
+    </row>
+    <row r="1190" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1190" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1190" s="20">
+        <v>1438</v>
+      </c>
+      <c r="D1190" s="20">
+        <v>1432</v>
+      </c>
+      <c r="E1190" s="20">
+        <f t="shared" ref="E1190:E1197" si="453">C1190-D1190</f>
+        <v>6</v>
+      </c>
+      <c r="F1190" s="3">
+        <f t="shared" ref="F1190:F1197" si="454">D1190/C1190</f>
+        <v>0.99582753824756609</v>
+      </c>
+      <c r="G1190" s="2">
+        <v>5</v>
+      </c>
+      <c r="H1190" s="4">
+        <f t="shared" si="452"/>
+        <v>286.39999999999998</v>
+      </c>
+      <c r="I1190" s="10">
+        <v>46121</v>
+      </c>
+      <c r="J1190" s="17">
+        <v>8</v>
+      </c>
+      <c r="K1190" s="17"/>
+      <c r="L1190" s="17"/>
+      <c r="M1190" s="17">
+        <v>9</v>
+      </c>
+      <c r="N1190" s="17"/>
+    </row>
+    <row r="1191" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1191" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1191" s="6">
+        <v>574</v>
+      </c>
+      <c r="D1191" s="6">
+        <v>521</v>
+      </c>
+      <c r="E1191" s="2">
+        <f t="shared" si="453"/>
+        <v>53</v>
+      </c>
+      <c r="F1191" s="3">
+        <f t="shared" si="454"/>
+        <v>0.90766550522648082</v>
+      </c>
+      <c r="G1191" s="2">
+        <v>9</v>
+      </c>
+      <c r="H1191" s="4">
+        <f t="shared" si="452"/>
+        <v>57.888888888888886</v>
+      </c>
+      <c r="I1191" s="10">
+        <v>46121</v>
+      </c>
+      <c r="J1191" s="17">
+        <v>1</v>
+      </c>
+      <c r="K1191" s="17"/>
+      <c r="L1191" s="17"/>
+      <c r="M1191" s="17"/>
+      <c r="N1191" s="17">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1192" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1192" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1192" s="2">
+        <v>37</v>
+      </c>
+      <c r="D1192" s="2">
+        <v>37</v>
+      </c>
+      <c r="E1192" s="2">
+        <f t="shared" si="453"/>
+        <v>0</v>
+      </c>
+      <c r="F1192" s="3">
+        <f t="shared" si="454"/>
+        <v>1</v>
+      </c>
+      <c r="G1192" s="2">
+        <v>9</v>
+      </c>
+      <c r="H1192" s="4">
+        <f t="shared" si="452"/>
+        <v>4.1111111111111107</v>
+      </c>
+      <c r="I1192" s="10">
+        <v>46121</v>
+      </c>
+      <c r="J1192" s="17"/>
+      <c r="K1192" s="17"/>
+      <c r="L1192" s="17"/>
+      <c r="M1192" s="17"/>
+      <c r="N1192" s="17"/>
+    </row>
+    <row r="1193" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1193" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1193" s="6">
+        <f>582+25+248</f>
+        <v>855</v>
+      </c>
+      <c r="D1193" s="99">
+        <f>578+248</f>
+        <v>826</v>
+      </c>
+      <c r="E1193" s="2">
+        <f t="shared" si="453"/>
+        <v>29</v>
+      </c>
+      <c r="F1193" s="3">
+        <f t="shared" si="454"/>
+        <v>0.96608187134502921</v>
+      </c>
+      <c r="G1193" s="6">
+        <v>10</v>
+      </c>
+      <c r="H1193" s="4">
+        <f t="shared" si="452"/>
+        <v>82.6</v>
+      </c>
+      <c r="I1193" s="10">
+        <v>46121</v>
+      </c>
+      <c r="J1193" s="17"/>
+      <c r="K1193" s="17"/>
+      <c r="L1193" s="17"/>
+      <c r="M1193" s="17"/>
+      <c r="N1193" s="17"/>
+    </row>
+    <row r="1194" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1194" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1194" s="20">
+        <v>566</v>
+      </c>
+      <c r="D1194" s="20">
+        <v>513</v>
+      </c>
+      <c r="E1194" s="2">
+        <f t="shared" si="453"/>
+        <v>53</v>
+      </c>
+      <c r="F1194" s="3">
+        <f t="shared" si="454"/>
+        <v>0.90636042402826855</v>
+      </c>
+      <c r="G1194" s="6">
+        <v>9</v>
+      </c>
+      <c r="H1194" s="4">
+        <f t="shared" si="452"/>
+        <v>57</v>
+      </c>
+      <c r="I1194" s="10">
+        <v>46121</v>
+      </c>
+      <c r="J1194" s="17">
+        <v>1</v>
+      </c>
+      <c r="K1194" s="17">
+        <v>11</v>
+      </c>
+      <c r="L1194" s="17"/>
+      <c r="M1194" s="17"/>
+      <c r="N1194" s="17"/>
+    </row>
+    <row r="1195" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1195" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1195" s="20">
+        <v>364</v>
+      </c>
+      <c r="D1195" s="20">
+        <v>358</v>
+      </c>
+      <c r="E1195" s="2">
+        <f t="shared" si="453"/>
+        <v>6</v>
+      </c>
+      <c r="F1195" s="3">
+        <f t="shared" si="454"/>
+        <v>0.98351648351648346</v>
+      </c>
+      <c r="G1195" s="6">
+        <v>16</v>
+      </c>
+      <c r="H1195" s="4">
+        <f t="shared" si="452"/>
+        <v>22.375</v>
+      </c>
+      <c r="I1195" s="10">
+        <v>46121</v>
+      </c>
+      <c r="J1195" s="17">
+        <v>1</v>
+      </c>
+      <c r="K1195" s="17"/>
+      <c r="L1195" s="17"/>
+      <c r="M1195" s="17"/>
+      <c r="N1195" s="17"/>
+      <c r="O1195">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="1196" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1196" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1196" s="2">
+        <v>787</v>
+      </c>
+      <c r="D1196" s="6">
+        <v>779</v>
+      </c>
+      <c r="E1196" s="2">
+        <f t="shared" si="453"/>
+        <v>8</v>
+      </c>
+      <c r="F1196" s="3">
+        <f t="shared" si="454"/>
+        <v>0.9898348157560356</v>
+      </c>
+      <c r="G1196" s="6">
+        <v>4</v>
+      </c>
+      <c r="H1196" s="4">
+        <f t="shared" ref="H1196:H1203" si="455">D1196/G1196</f>
+        <v>194.75</v>
+      </c>
+      <c r="I1196" s="10">
+        <v>46121</v>
+      </c>
+      <c r="J1196" s="17"/>
+      <c r="K1196" s="17"/>
+      <c r="L1196" s="17">
+        <v>8</v>
+      </c>
+      <c r="M1196" s="17"/>
+      <c r="N1196" s="17">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="1197" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1197" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1197" s="2">
+        <v>584</v>
+      </c>
+      <c r="D1197" s="6">
+        <v>578</v>
+      </c>
+      <c r="E1197" s="2">
+        <f t="shared" si="453"/>
+        <v>6</v>
+      </c>
+      <c r="F1197" s="3">
+        <f t="shared" si="454"/>
+        <v>0.98972602739726023</v>
+      </c>
+      <c r="G1197" s="6">
+        <v>2</v>
+      </c>
+      <c r="H1197" s="4">
+        <f t="shared" si="455"/>
+        <v>289</v>
+      </c>
+      <c r="I1197" s="10">
+        <v>46121</v>
+      </c>
+      <c r="J1197" s="17"/>
+      <c r="K1197" s="17"/>
+      <c r="L1197" s="17"/>
+      <c r="M1197" s="17"/>
+      <c r="N1197" s="17"/>
+    </row>
+    <row r="1198" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1198" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1198" s="20">
+        <v>623</v>
+      </c>
+      <c r="D1198" s="20">
+        <v>621</v>
+      </c>
+      <c r="E1198" s="20">
+        <f t="shared" ref="E1198:E1205" si="456">C1198-D1198</f>
+        <v>2</v>
+      </c>
+      <c r="F1198" s="3">
+        <f t="shared" ref="F1198:F1205" si="457">D1198/C1198</f>
+        <v>0.9967897271268058</v>
+      </c>
+      <c r="G1198" s="2">
+        <v>5</v>
+      </c>
+      <c r="H1198" s="4">
+        <f t="shared" si="455"/>
+        <v>124.2</v>
+      </c>
+      <c r="I1198" s="10">
+        <v>46122</v>
+      </c>
+      <c r="J1198" s="17"/>
+      <c r="K1198" s="17"/>
+      <c r="L1198" s="17"/>
+      <c r="M1198" s="17">
+        <v>7</v>
+      </c>
+      <c r="N1198" s="17"/>
+    </row>
+    <row r="1199" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1199" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1199" s="6">
+        <v>595</v>
+      </c>
+      <c r="D1199" s="6">
+        <v>578</v>
+      </c>
+      <c r="E1199" s="2">
+        <f t="shared" si="456"/>
+        <v>17</v>
+      </c>
+      <c r="F1199" s="3">
+        <f t="shared" si="457"/>
+        <v>0.97142857142857142</v>
+      </c>
+      <c r="G1199" s="2">
+        <v>9</v>
+      </c>
+      <c r="H1199" s="4">
+        <f t="shared" si="455"/>
+        <v>64.222222222222229</v>
+      </c>
+      <c r="I1199" s="10">
+        <v>46122</v>
+      </c>
+      <c r="J1199" s="17">
+        <v>3</v>
+      </c>
+      <c r="K1199" s="17"/>
+      <c r="L1199" s="17"/>
+      <c r="M1199" s="17"/>
+      <c r="N1199" s="17">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="1200" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1200" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1200" s="2">
+        <v>74</v>
+      </c>
+      <c r="D1200" s="2">
+        <v>71</v>
+      </c>
+      <c r="E1200" s="2">
+        <f t="shared" si="456"/>
+        <v>3</v>
+      </c>
+      <c r="F1200" s="3">
+        <f t="shared" si="457"/>
+        <v>0.95945945945945943</v>
+      </c>
+      <c r="G1200" s="2">
+        <v>9</v>
+      </c>
+      <c r="H1200" s="4">
+        <f t="shared" si="455"/>
+        <v>7.8888888888888893</v>
+      </c>
+      <c r="I1200" s="10">
+        <v>46122</v>
+      </c>
+      <c r="J1200" s="17"/>
+      <c r="K1200" s="17"/>
+      <c r="L1200" s="17"/>
+      <c r="M1200" s="17"/>
+      <c r="N1200" s="17"/>
+    </row>
+    <row r="1201" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1201" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1201" s="6">
+        <f>776+3+144</f>
+        <v>923</v>
+      </c>
+      <c r="D1201" s="99">
+        <f>614+1+88</f>
+        <v>703</v>
+      </c>
+      <c r="E1201" s="2">
+        <f t="shared" si="456"/>
+        <v>220</v>
+      </c>
+      <c r="F1201" s="3">
+        <f t="shared" si="457"/>
+        <v>0.76164680390032502</v>
+      </c>
+      <c r="G1201" s="6">
+        <v>10</v>
+      </c>
+      <c r="H1201" s="4">
+        <f t="shared" si="455"/>
+        <v>70.3</v>
+      </c>
+      <c r="I1201" s="10">
+        <v>46122</v>
+      </c>
+      <c r="J1201" s="17">
+        <v>27</v>
+      </c>
+      <c r="K1201" s="17"/>
+      <c r="L1201" s="17"/>
+      <c r="M1201" s="17"/>
+      <c r="N1201" s="17"/>
+    </row>
+    <row r="1202" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1202" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1202" s="20">
+        <v>1168</v>
+      </c>
+      <c r="D1202" s="20">
+        <v>1164</v>
+      </c>
+      <c r="E1202" s="2">
+        <f t="shared" si="456"/>
+        <v>4</v>
+      </c>
+      <c r="F1202" s="3">
+        <f>D1202/C1202</f>
+        <v>0.99657534246575341</v>
+      </c>
+      <c r="G1202" s="6">
+        <v>9</v>
+      </c>
+      <c r="H1202" s="4">
+        <f t="shared" si="455"/>
+        <v>129.33333333333334</v>
+      </c>
+      <c r="I1202" s="10">
+        <v>46122</v>
+      </c>
+      <c r="J1202" s="17"/>
+      <c r="K1202" s="17">
+        <v>11</v>
+      </c>
+      <c r="L1202" s="17"/>
+      <c r="M1202" s="17"/>
+      <c r="N1202" s="17"/>
+    </row>
+    <row r="1203" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1203" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1203" s="20">
+        <v>313</v>
+      </c>
+      <c r="D1203" s="20">
+        <v>313</v>
+      </c>
+      <c r="E1203" s="2">
+        <f t="shared" si="456"/>
+        <v>0</v>
+      </c>
+      <c r="F1203" s="3">
+        <f t="shared" si="457"/>
+        <v>1</v>
+      </c>
+      <c r="G1203" s="6">
+        <v>16</v>
+      </c>
+      <c r="H1203" s="4">
+        <f t="shared" si="455"/>
+        <v>19.5625</v>
+      </c>
+      <c r="I1203" s="10">
+        <v>46122</v>
+      </c>
+      <c r="J1203" s="17"/>
+      <c r="K1203" s="17"/>
+      <c r="L1203" s="17"/>
+      <c r="M1203" s="17"/>
+      <c r="N1203" s="17"/>
+      <c r="O1203">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="1204" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1204" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1204" s="2">
+        <v>241</v>
+      </c>
+      <c r="D1204" s="6">
+        <v>235</v>
+      </c>
+      <c r="E1204" s="2">
+        <f t="shared" si="456"/>
+        <v>6</v>
+      </c>
+      <c r="F1204" s="3">
+        <f t="shared" si="457"/>
+        <v>0.975103734439834</v>
+      </c>
+      <c r="G1204" s="6">
+        <v>4</v>
+      </c>
+      <c r="H1204" s="4">
+        <f t="shared" ref="H1204:H1211" si="458">D1204/G1204</f>
+        <v>58.75</v>
+      </c>
+      <c r="I1204" s="10">
+        <v>46122</v>
+      </c>
+      <c r="J1204" s="17"/>
+      <c r="K1204" s="17"/>
+      <c r="L1204" s="17">
+        <v>11</v>
+      </c>
+      <c r="M1204" s="17"/>
+      <c r="N1204" s="17">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="1205" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1205" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1205" s="2">
+        <v>662</v>
+      </c>
+      <c r="D1205" s="6">
+        <v>624</v>
+      </c>
+      <c r="E1205" s="2">
+        <f t="shared" si="456"/>
+        <v>38</v>
+      </c>
+      <c r="F1205" s="3">
+        <f t="shared" si="457"/>
+        <v>0.94259818731117828</v>
+      </c>
+      <c r="G1205" s="6">
+        <v>2</v>
+      </c>
+      <c r="H1205" s="4">
+        <f t="shared" si="458"/>
+        <v>312</v>
+      </c>
+      <c r="I1205" s="10">
+        <v>46122</v>
+      </c>
+      <c r="J1205" s="17"/>
+      <c r="K1205" s="17"/>
+      <c r="L1205" s="17"/>
+      <c r="M1205" s="17"/>
+      <c r="N1205" s="17"/>
+    </row>
+    <row r="1206" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1206" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1206" s="20">
+        <v>173</v>
+      </c>
+      <c r="D1206" s="20">
+        <v>171</v>
+      </c>
+      <c r="E1206" s="20">
+        <f t="shared" ref="E1206:E1213" si="459">C1206-D1206</f>
+        <v>2</v>
+      </c>
+      <c r="F1206" s="3">
+        <f t="shared" ref="F1206:F1213" si="460">D1206/C1206</f>
+        <v>0.98843930635838151</v>
+      </c>
+      <c r="G1206" s="2">
+        <v>3</v>
+      </c>
+      <c r="H1206" s="4">
+        <f t="shared" si="458"/>
+        <v>57</v>
+      </c>
+      <c r="I1206" s="10">
+        <v>46125</v>
+      </c>
+      <c r="J1206" s="17">
+        <v>1</v>
+      </c>
+      <c r="K1206" s="17"/>
+      <c r="L1206" s="17"/>
+      <c r="M1206" s="17">
+        <v>8</v>
+      </c>
+      <c r="N1206" s="17"/>
+    </row>
+    <row r="1207" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1207" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1207" s="6">
+        <v>1228</v>
+      </c>
+      <c r="D1207" s="6">
+        <v>1110</v>
+      </c>
+      <c r="E1207" s="2">
+        <f t="shared" si="459"/>
+        <v>118</v>
+      </c>
+      <c r="F1207" s="3">
+        <f t="shared" si="460"/>
+        <v>0.90390879478827357</v>
+      </c>
+      <c r="G1207" s="2">
+        <v>9</v>
+      </c>
+      <c r="H1207" s="4">
+        <f t="shared" si="458"/>
+        <v>123.33333333333333</v>
+      </c>
+      <c r="I1207" s="10">
+        <v>46125</v>
+      </c>
+      <c r="J1207" s="17">
+        <v>3</v>
+      </c>
+      <c r="K1207" s="17"/>
+      <c r="L1207" s="17"/>
+      <c r="M1207" s="17"/>
+      <c r="N1207" s="17">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="1208" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1208" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1208" s="2">
+        <v>234</v>
+      </c>
+      <c r="D1208" s="2">
+        <v>232</v>
+      </c>
+      <c r="E1208" s="2">
+        <f t="shared" si="459"/>
+        <v>2</v>
+      </c>
+      <c r="F1208" s="3">
+        <f t="shared" si="460"/>
+        <v>0.99145299145299148</v>
+      </c>
+      <c r="G1208" s="2">
+        <v>9</v>
+      </c>
+      <c r="H1208" s="4">
+        <f t="shared" si="458"/>
+        <v>25.777777777777779</v>
+      </c>
+      <c r="I1208" s="10">
+        <v>46125</v>
+      </c>
+      <c r="J1208" s="17"/>
+      <c r="K1208" s="17"/>
+      <c r="L1208" s="17"/>
+      <c r="M1208" s="17"/>
+      <c r="N1208" s="17"/>
+    </row>
+    <row r="1209" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1209" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1209" s="6">
+        <f>525+12+572</f>
+        <v>1109</v>
+      </c>
+      <c r="D1209" s="99">
+        <f>189+488</f>
+        <v>677</v>
+      </c>
+      <c r="E1209" s="2">
+        <f t="shared" si="459"/>
+        <v>432</v>
+      </c>
+      <c r="F1209" s="3">
+        <f t="shared" si="460"/>
+        <v>0.61045987376014432</v>
+      </c>
+      <c r="G1209" s="6">
+        <v>10</v>
+      </c>
+      <c r="H1209" s="4">
+        <f t="shared" si="458"/>
+        <v>67.7</v>
+      </c>
+      <c r="I1209" s="10">
+        <v>46125</v>
+      </c>
+      <c r="J1209" s="17">
+        <v>8</v>
+      </c>
+      <c r="K1209" s="17"/>
+      <c r="L1209" s="17"/>
+      <c r="M1209" s="17"/>
+      <c r="N1209" s="17"/>
+    </row>
+    <row r="1210" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1210" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1210" s="20">
+        <v>566</v>
+      </c>
+      <c r="D1210" s="20">
+        <v>513</v>
+      </c>
+      <c r="E1210" s="2">
+        <f t="shared" si="459"/>
+        <v>53</v>
+      </c>
+      <c r="F1210" s="3">
+        <f t="shared" si="460"/>
+        <v>0.90636042402826855</v>
+      </c>
+      <c r="G1210" s="6">
+        <v>10</v>
+      </c>
+      <c r="H1210" s="4">
+        <f t="shared" si="458"/>
+        <v>51.3</v>
+      </c>
+      <c r="I1210" s="10">
+        <v>46125</v>
+      </c>
+      <c r="J1210" s="17">
+        <v>4</v>
+      </c>
+      <c r="K1210" s="17">
+        <v>9</v>
+      </c>
+      <c r="L1210" s="17"/>
+      <c r="M1210" s="17"/>
+      <c r="N1210" s="17"/>
+    </row>
+    <row r="1211" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1211" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1211" s="20">
+        <v>272</v>
+      </c>
+      <c r="D1211" s="20">
+        <v>271</v>
+      </c>
+      <c r="E1211" s="2">
+        <f t="shared" si="459"/>
+        <v>1</v>
+      </c>
+      <c r="F1211" s="3">
+        <f t="shared" si="460"/>
+        <v>0.99632352941176472</v>
+      </c>
+      <c r="G1211" s="6">
+        <v>18</v>
+      </c>
+      <c r="H1211" s="4">
+        <f t="shared" si="458"/>
+        <v>15.055555555555555</v>
+      </c>
+      <c r="I1211" s="10">
+        <v>46125</v>
+      </c>
+      <c r="J1211" s="17"/>
+      <c r="K1211" s="17"/>
+      <c r="L1211" s="17"/>
+      <c r="M1211" s="17"/>
+      <c r="N1211" s="17"/>
+      <c r="O1211">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="1212" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1212" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1212" s="2">
+        <v>35</v>
+      </c>
+      <c r="D1212" s="6">
+        <v>35</v>
+      </c>
+      <c r="E1212" s="2">
+        <f t="shared" si="459"/>
+        <v>0</v>
+      </c>
+      <c r="F1212" s="3">
+        <f t="shared" si="460"/>
+        <v>1</v>
+      </c>
+      <c r="G1212" s="6">
+        <v>4</v>
+      </c>
+      <c r="H1212" s="4">
+        <f t="shared" ref="H1212:H1219" si="461">D1212/G1212</f>
+        <v>8.75</v>
+      </c>
+      <c r="I1212" s="10">
+        <v>46125</v>
+      </c>
+      <c r="J1212" s="17"/>
+      <c r="K1212" s="17"/>
+      <c r="L1212" s="17">
+        <v>5</v>
+      </c>
+      <c r="M1212" s="17"/>
+      <c r="N1212" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1213" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1213" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1213" s="2">
+        <v>435</v>
+      </c>
+      <c r="D1213" s="6">
+        <v>435</v>
+      </c>
+      <c r="E1213" s="2">
+        <f t="shared" si="459"/>
+        <v>0</v>
+      </c>
+      <c r="F1213" s="3">
+        <f t="shared" si="460"/>
+        <v>1</v>
+      </c>
+      <c r="G1213" s="6">
+        <v>2</v>
+      </c>
+      <c r="H1213" s="4">
+        <f t="shared" si="461"/>
+        <v>217.5</v>
+      </c>
+      <c r="I1213" s="10">
+        <v>46125</v>
+      </c>
+      <c r="J1213" s="17"/>
+      <c r="K1213" s="17"/>
+      <c r="L1213" s="17"/>
+      <c r="M1213" s="17"/>
+      <c r="N1213" s="17"/>
+    </row>
+    <row r="1214" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1214" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1214" s="20">
+        <v>38</v>
+      </c>
+      <c r="D1214" s="20">
+        <v>38</v>
+      </c>
+      <c r="E1214" s="20">
+        <f t="shared" ref="E1214:E1221" si="462">C1214-D1214</f>
+        <v>0</v>
+      </c>
+      <c r="F1214" s="3">
+        <f t="shared" ref="F1214:F1221" si="463">D1214/C1214</f>
+        <v>1</v>
+      </c>
+      <c r="G1214" s="2">
+        <v>3</v>
+      </c>
+      <c r="H1214" s="4">
+        <f t="shared" si="461"/>
+        <v>12.666666666666666</v>
+      </c>
+      <c r="I1214" s="10">
+        <v>46126</v>
+      </c>
+      <c r="J1214" s="17">
+        <v>2</v>
+      </c>
+      <c r="K1214" s="17"/>
+      <c r="L1214" s="17"/>
+      <c r="M1214" s="17">
+        <v>6</v>
+      </c>
+      <c r="N1214" s="17"/>
+    </row>
+    <row r="1215" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1215" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1215" s="6">
+        <v>648</v>
+      </c>
+      <c r="D1215" s="6">
+        <v>646</v>
+      </c>
+      <c r="E1215" s="2">
+        <f t="shared" si="462"/>
+        <v>2</v>
+      </c>
+      <c r="F1215" s="3">
+        <f t="shared" si="463"/>
+        <v>0.99691358024691357</v>
+      </c>
+      <c r="G1215" s="2">
+        <v>9</v>
+      </c>
+      <c r="H1215" s="4">
+        <f t="shared" si="461"/>
+        <v>71.777777777777771</v>
+      </c>
+      <c r="I1215" s="10">
+        <v>46126</v>
+      </c>
+      <c r="J1215" s="17">
+        <v>13</v>
+      </c>
+      <c r="K1215" s="17"/>
+      <c r="L1215" s="17"/>
+      <c r="M1215" s="17"/>
+      <c r="N1215" s="17">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="1216" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1216" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1216" s="2">
+        <v>281</v>
+      </c>
+      <c r="D1216" s="2">
+        <v>281</v>
+      </c>
+      <c r="E1216" s="2">
+        <f t="shared" si="462"/>
+        <v>0</v>
+      </c>
+      <c r="F1216" s="3">
+        <f t="shared" si="463"/>
+        <v>1</v>
+      </c>
+      <c r="G1216" s="2">
+        <v>9</v>
+      </c>
+      <c r="H1216" s="4">
+        <f t="shared" si="461"/>
+        <v>31.222222222222221</v>
+      </c>
+      <c r="I1216" s="10">
+        <v>46126</v>
+      </c>
+      <c r="J1216" s="17"/>
+      <c r="K1216" s="17"/>
+      <c r="L1216" s="17"/>
+      <c r="M1216" s="17"/>
+      <c r="N1216" s="17"/>
+    </row>
+    <row r="1217" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1217" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1217" s="6">
+        <f>780+92</f>
+        <v>872</v>
+      </c>
+      <c r="D1217" s="99">
+        <f>432+2</f>
+        <v>434</v>
+      </c>
+      <c r="E1217" s="2">
+        <f t="shared" si="462"/>
+        <v>438</v>
+      </c>
+      <c r="F1217" s="3">
+        <f t="shared" si="463"/>
+        <v>0.49770642201834864</v>
+      </c>
+      <c r="G1217" s="6">
+        <v>10</v>
+      </c>
+      <c r="H1217" s="4">
+        <f t="shared" si="461"/>
+        <v>43.4</v>
+      </c>
+      <c r="I1217" s="10">
+        <v>46126</v>
+      </c>
+      <c r="J1217" s="17"/>
+      <c r="K1217" s="17"/>
+      <c r="L1217" s="17"/>
+      <c r="M1217" s="17"/>
+      <c r="N1217" s="17"/>
+    </row>
+    <row r="1218" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1218" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1218" s="20">
+        <v>1304</v>
+      </c>
+      <c r="D1218" s="20">
+        <v>1140</v>
+      </c>
+      <c r="E1218" s="2">
+        <f t="shared" si="462"/>
+        <v>164</v>
+      </c>
+      <c r="F1218" s="3">
+        <f t="shared" si="463"/>
+        <v>0.87423312883435578</v>
+      </c>
+      <c r="G1218" s="6">
+        <v>10</v>
+      </c>
+      <c r="H1218" s="4">
+        <f t="shared" si="461"/>
+        <v>114</v>
+      </c>
+      <c r="I1218" s="10">
+        <v>46126</v>
+      </c>
+      <c r="J1218" s="17">
+        <v>5</v>
+      </c>
+      <c r="K1218" s="17">
+        <v>11</v>
+      </c>
+      <c r="L1218" s="17"/>
+      <c r="M1218" s="17"/>
+      <c r="N1218" s="17"/>
+    </row>
+    <row r="1219" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1219" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1219" s="20">
+        <v>287</v>
+      </c>
+      <c r="D1219" s="20">
+        <v>267</v>
+      </c>
+      <c r="E1219" s="2">
+        <f t="shared" si="462"/>
+        <v>20</v>
+      </c>
+      <c r="F1219" s="3">
+        <f t="shared" si="463"/>
+        <v>0.93031358885017423</v>
+      </c>
+      <c r="G1219" s="6">
+        <v>18</v>
+      </c>
+      <c r="H1219" s="4">
+        <f t="shared" si="461"/>
+        <v>14.833333333333334</v>
+      </c>
+      <c r="I1219" s="10">
+        <v>46126</v>
+      </c>
+      <c r="J1219" s="17">
+        <v>1</v>
+      </c>
+      <c r="K1219" s="17"/>
+      <c r="L1219" s="17"/>
+      <c r="M1219" s="17"/>
+      <c r="N1219" s="17"/>
+      <c r="O1219">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="1220" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1220" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1220" s="2">
+        <v>523</v>
+      </c>
+      <c r="D1220" s="6">
+        <v>523</v>
+      </c>
+      <c r="E1220" s="2">
+        <f t="shared" si="462"/>
+        <v>0</v>
+      </c>
+      <c r="F1220" s="3">
+        <f t="shared" si="463"/>
+        <v>1</v>
+      </c>
+      <c r="G1220" s="6">
+        <v>4</v>
+      </c>
+      <c r="H1220" s="4">
+        <f t="shared" ref="H1220:H1221" si="464">D1220/G1220</f>
+        <v>130.75</v>
+      </c>
+      <c r="I1220" s="10">
+        <v>46126</v>
+      </c>
+      <c r="J1220" s="17"/>
+      <c r="K1220" s="17"/>
+      <c r="L1220" s="17">
+        <v>11</v>
+      </c>
+      <c r="M1220" s="17"/>
+      <c r="N1220" s="17">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="1221" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1221" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1221" s="2">
+        <v>626</v>
+      </c>
+      <c r="D1221" s="6">
+        <v>207</v>
+      </c>
+      <c r="E1221" s="2">
+        <f t="shared" si="462"/>
+        <v>419</v>
+      </c>
+      <c r="F1221" s="3">
+        <f t="shared" si="463"/>
+        <v>0.33067092651757191</v>
+      </c>
+      <c r="G1221" s="6">
+        <v>2</v>
+      </c>
+      <c r="H1221" s="4">
+        <f t="shared" si="464"/>
+        <v>103.5</v>
+      </c>
+      <c r="I1221" s="10">
+        <v>46126</v>
+      </c>
+      <c r="J1221" s="17"/>
+      <c r="K1221" s="17"/>
+      <c r="L1221" s="17"/>
+      <c r="M1221" s="17"/>
+      <c r="N1221" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -39542,7 +41049,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E86DB14F-1817-4DEB-B8E4-6703848319FA}">
   <sheetPr codeName="Sayfa2"/>
-  <dimension ref="A1:D146"/>
+  <dimension ref="A1:D150"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.1640625" bestFit="1" customWidth="1"/>
@@ -41725,6 +43232,66 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
+    <row r="147" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A147" s="18">
+        <v>46121</v>
+      </c>
+      <c r="B147" s="113" t="s">
+        <v>120</v>
+      </c>
+      <c r="C147">
+        <v>6</v>
+      </c>
+      <c r="D147" s="19">
+        <f>C147/6</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A148" s="18">
+        <v>46125</v>
+      </c>
+      <c r="B148" s="114" t="s">
+        <v>140</v>
+      </c>
+      <c r="C148">
+        <v>1</v>
+      </c>
+      <c r="D148" s="19">
+        <f>C148/1</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A149" s="18">
+        <v>46126</v>
+      </c>
+      <c r="B149" s="115" t="s">
+        <v>141</v>
+      </c>
+      <c r="C149">
+        <v>16</v>
+      </c>
+      <c r="D149" s="19">
+        <f>C149/20</f>
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A150" s="18">
+        <v>46126</v>
+      </c>
+      <c r="B150" s="115" t="s">
+        <v>142</v>
+      </c>
+      <c r="C150">
+        <v>4</v>
+      </c>
+      <c r="D150" s="19">
+        <f>C150/20</f>
+        <v>0.2</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D124" xr:uid="{E86DB14F-1817-4DEB-B8E4-6703848319FA}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>